<commit_message>
Update decision log for terminology-unification phase kickoff
</commit_message>
<xml_diff>
--- a/docs/IO_from_order_to_invoice_revised_v_2.xlsx
+++ b/docs/IO_from_order_to_invoice_revised_v_2.xlsx
@@ -9,11 +9,11 @@
   </bookViews>
   <sheets>
     <sheet name="EntryMethod_Rules" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Sheet2" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="main" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="permission_matrix" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$2:$U$94</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">main!$A$2:$U$94</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1712" uniqueCount="679">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1791" uniqueCount="687">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -2319,89 +2319,114 @@
     <t xml:space="preserve">print template</t>
   </si>
   <si>
-    <t xml:space="preserve">2) Entry Method（固定語彙）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">manual（手入力）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lookup_select（マスタ検索して選択）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">auto_default（デフォルト自動補完）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">auth_context（ログインユーザー/権限から確定）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">system_timestamp（システム時刻）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rule_engine（配賦/判定ロジック）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">calculated（数式計算）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">api_response（レスポンス専用）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">print_render（帳票レンダリング専用）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n/a（validation/output_rule用）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Direction（固定語彙）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ユーザー/APIから受け付ける値 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">他データ/認証主体/ルールから決まる値 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">システムが新規発行する値（ID/番号） </t>
-  </si>
-  <si>
-    <t xml:space="preserve">APIレスポンスや帳票出力で返す値 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">値そのものではなく検証ルール</t>
-  </si>
-  <si>
-    <t xml:space="preserve">表示/非表示など出力制御ルール</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4) 置換ルール（既存値→統一値）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">derived/input or input/derived →</t>
-  </si>
-  <si>
-    <t xml:space="preserve">原則 input（自動補完はEntry Methodで表現） </t>
-  </si>
-  <si>
-    <t xml:space="preserve">derived/editable → derived</t>
-  </si>
-  <si>
-    <t xml:space="preserve">search box → Directionは input、Entry Methodは lookup_select</t>
-  </si>
-  <si>
-    <t xml:space="preserve">output rule → output_rule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI/API request など境界説明は Entry Method ではなく I/O Boundary 列へ移す</t>
+    <t xml:space="preserve">role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scope_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_view_order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_view_invoice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_cancel_order_new</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_cancel_order_confirmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_cancel_order_allocated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_cancel_order_purchased</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_cancel_order_shipped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_cancel_order_invoiced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_cancel_line_uninvoiced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_cancel_line_partially_invoiced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_cancel_line_invoiced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_cancel_line_when_invoice_draft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_reset_invoice_to_draft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">require_reason_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">require_note_on_policy_exception</t>
+  </si>
+  <si>
+    <t xml:space="preserve">notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">global</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full authority</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> invoiced order direct cancel is blocked (use reset/credit flow)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OrderEntry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">own</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can cancel own orders only in new status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assigned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can cancel assigned orders/lines</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> purchased+ and shipped order cancel not allowed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No cancel permission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No direct cancel permission (request via operator)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
     <numFmt numFmtId="166" formatCode="General"/>
+    <numFmt numFmtId="167" formatCode="@"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -2465,12 +2490,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF999999"/>
+        <bgColor rgb="FF808080"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -2513,7 +2544,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2558,6 +2589,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2574,15 +2617,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2595,7 +2646,15 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF999999"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2685,7 +2744,7 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF6B5E9B"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF999999"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF3FAF46"/>
       <rgbColor rgb="FF003300"/>
@@ -3275,7 +3334,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="true">
+  <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:U95"/>
@@ -3384,7 +3443,7 @@
       <c r="T2" s="3"/>
       <c r="U2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
         <v>101</v>
       </c>
@@ -3439,7 +3498,7 @@
       <c r="T3" s="5"/>
       <c r="U3" s="8"/>
     </row>
-    <row r="4" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
         <v>101</v>
       </c>
@@ -3492,7 +3551,7 @@
       <c r="T4" s="5"/>
       <c r="U4" s="8"/>
     </row>
-    <row r="5" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>101</v>
       </c>
@@ -3545,7 +3604,7 @@
       <c r="T5" s="5"/>
       <c r="U5" s="8"/>
     </row>
-    <row r="6" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>101</v>
       </c>
@@ -3601,7 +3660,7 @@
       <c r="T6" s="5"/>
       <c r="U6" s="8"/>
     </row>
-    <row r="7" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>101</v>
       </c>
@@ -3662,7 +3721,7 @@
       <c r="T7" s="5"/>
       <c r="U7" s="8"/>
     </row>
-    <row r="8" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
         <v>101</v>
       </c>
@@ -3715,7 +3774,7 @@
       <c r="T8" s="5"/>
       <c r="U8" s="8"/>
     </row>
-    <row r="9" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
         <v>101</v>
       </c>
@@ -3827,7 +3886,7 @@
       <c r="T10" s="5"/>
       <c r="U10" s="8"/>
     </row>
-    <row r="11" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>101</v>
       </c>
@@ -3888,7 +3947,7 @@
       <c r="T11" s="5"/>
       <c r="U11" s="8"/>
     </row>
-    <row r="12" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
         <v>101</v>
       </c>
@@ -3949,7 +4008,7 @@
       <c r="T12" s="5"/>
       <c r="U12" s="8"/>
     </row>
-    <row r="13" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
         <v>101</v>
       </c>
@@ -4008,7 +4067,7 @@
       <c r="T13" s="5"/>
       <c r="U13" s="8"/>
     </row>
-    <row r="14" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
         <v>101</v>
       </c>
@@ -4064,7 +4123,7 @@
       <c r="T14" s="5"/>
       <c r="U14" s="8"/>
     </row>
-    <row r="15" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
         <v>101</v>
       </c>
@@ -4120,7 +4179,7 @@
       <c r="T15" s="5"/>
       <c r="U15" s="8"/>
     </row>
-    <row r="16" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
         <v>101</v>
       </c>
@@ -4176,7 +4235,7 @@
       <c r="T16" s="5"/>
       <c r="U16" s="8"/>
     </row>
-    <row r="17" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
         <v>101</v>
       </c>
@@ -4232,7 +4291,7 @@
       <c r="T17" s="5"/>
       <c r="U17" s="8"/>
     </row>
-    <row r="18" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
         <v>101</v>
       </c>
@@ -4288,7 +4347,7 @@
       <c r="T18" s="5"/>
       <c r="U18" s="8"/>
     </row>
-    <row r="19" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
         <v>209</v>
       </c>
@@ -4344,7 +4403,7 @@
       <c r="T19" s="5"/>
       <c r="U19" s="8"/>
     </row>
-    <row r="20" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
         <v>209</v>
       </c>
@@ -4385,7 +4444,7 @@
       <c r="T20" s="5"/>
       <c r="U20" s="8"/>
     </row>
-    <row r="21" customFormat="false" ht="12" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
         <v>209</v>
       </c>
@@ -4441,7 +4500,7 @@
       <c r="T21" s="5"/>
       <c r="U21" s="8"/>
     </row>
-    <row r="22" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
         <v>209</v>
       </c>
@@ -4497,7 +4556,7 @@
       <c r="T22" s="5"/>
       <c r="U22" s="8"/>
     </row>
-    <row r="23" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
         <v>209</v>
       </c>
@@ -4553,7 +4612,7 @@
       <c r="T23" s="5"/>
       <c r="U23" s="8"/>
     </row>
-    <row r="24" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
         <v>209</v>
       </c>
@@ -4609,7 +4668,7 @@
       <c r="T24" s="5"/>
       <c r="U24" s="8"/>
     </row>
-    <row r="25" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
         <v>209</v>
       </c>
@@ -4665,7 +4724,7 @@
       <c r="T25" s="5"/>
       <c r="U25" s="8"/>
     </row>
-    <row r="26" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
         <v>209</v>
       </c>
@@ -4721,7 +4780,7 @@
       <c r="T26" s="5"/>
       <c r="U26" s="8"/>
     </row>
-    <row r="27" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
         <v>209</v>
       </c>
@@ -4774,7 +4833,7 @@
       <c r="T27" s="5"/>
       <c r="U27" s="8"/>
     </row>
-    <row r="28" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
         <v>209</v>
       </c>
@@ -4883,7 +4942,7 @@
       <c r="T29" s="5"/>
       <c r="U29" s="8"/>
     </row>
-    <row r="30" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
         <v>267</v>
       </c>
@@ -4933,7 +4992,7 @@
       <c r="T30" s="5"/>
       <c r="U30" s="8"/>
     </row>
-    <row r="31" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
         <v>267</v>
       </c>
@@ -4983,7 +5042,7 @@
       <c r="T31" s="5"/>
       <c r="U31" s="8"/>
     </row>
-    <row r="32" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
         <v>267</v>
       </c>
@@ -5034,7 +5093,7 @@
       <c r="T32" s="5"/>
       <c r="U32" s="8"/>
     </row>
-    <row r="33" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
         <v>285</v>
       </c>
@@ -5084,7 +5143,7 @@
       <c r="T33" s="5"/>
       <c r="U33" s="8"/>
     </row>
-    <row r="34" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
         <v>288</v>
       </c>
@@ -5140,7 +5199,7 @@
       <c r="T34" s="5"/>
       <c r="U34" s="8"/>
     </row>
-    <row r="35" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
         <v>288</v>
       </c>
@@ -5196,7 +5255,7 @@
       <c r="T35" s="5"/>
       <c r="U35" s="8"/>
     </row>
-    <row r="36" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
         <v>288</v>
       </c>
@@ -5252,7 +5311,7 @@
       <c r="T36" s="5"/>
       <c r="U36" s="8"/>
     </row>
-    <row r="37" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
         <v>246</v>
       </c>
@@ -5313,7 +5372,7 @@
       <c r="T37" s="5"/>
       <c r="U37" s="8"/>
     </row>
-    <row r="38" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
         <v>246</v>
       </c>
@@ -5375,50 +5434,50 @@
       <c r="U38" s="8"/>
     </row>
     <row r="39" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="11" t="s">
         <v>246</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="11" t="s">
         <v>260</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D39" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="E39" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5" t="s">
+      <c r="F39" s="11"/>
+      <c r="G39" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="H39" s="5" t="s">
+      <c r="H39" s="11" t="s">
         <v>328</v>
       </c>
-      <c r="I39" s="5" t="s">
+      <c r="I39" s="11" t="s">
         <v>329</v>
       </c>
-      <c r="J39" s="5" t="s">
+      <c r="J39" s="11" t="s">
         <v>329</v>
       </c>
-      <c r="K39" s="5" t="s">
+      <c r="K39" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="L39" s="2" t="s">
+      <c r="L39" s="13" t="s">
         <v>330</v>
       </c>
-      <c r="M39" s="5" t="s">
+      <c r="M39" s="11" t="s">
         <v>264</v>
       </c>
-      <c r="N39" s="5" t="s">
+      <c r="N39" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="O39" s="5" t="s">
+      <c r="O39" s="11" t="s">
         <v>332</v>
       </c>
-      <c r="P39" s="2" t="s">
+      <c r="P39" s="13" t="s">
         <v>39</v>
       </c>
       <c r="Q39" s="5" t="s">
@@ -5433,7 +5492,7 @@
       <c r="T39" s="5"/>
       <c r="U39" s="8"/>
     </row>
-    <row r="40" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
         <v>246</v>
       </c>
@@ -5494,7 +5553,7 @@
       <c r="T40" s="5"/>
       <c r="U40" s="8"/>
     </row>
-    <row r="41" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
         <v>246</v>
       </c>
@@ -5553,7 +5612,7 @@
       <c r="T41" s="5"/>
       <c r="U41" s="8"/>
     </row>
-    <row r="42" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
         <v>246</v>
       </c>
@@ -5600,7 +5659,7 @@
       <c r="T42" s="5"/>
       <c r="U42" s="8"/>
     </row>
-    <row r="43" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
         <v>246</v>
       </c>
@@ -5610,7 +5669,7 @@
       <c r="C43" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="D43" s="11" t="s">
+      <c r="D43" s="14" t="s">
         <v>352</v>
       </c>
       <c r="E43" s="5" t="s">
@@ -5656,7 +5715,7 @@
       <c r="T43" s="5"/>
       <c r="U43" s="8"/>
     </row>
-    <row r="44" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
         <v>246</v>
       </c>
@@ -5679,7 +5738,7 @@
       <c r="H44" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="I44" s="12" t="b">
+      <c r="I44" s="15" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -5716,7 +5775,7 @@
       <c r="T44" s="5"/>
       <c r="U44" s="8"/>
     </row>
-    <row r="45" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
         <v>246</v>
       </c>
@@ -5772,7 +5831,7 @@
       <c r="T45" s="5"/>
       <c r="U45" s="8"/>
     </row>
-    <row r="46" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
         <v>246</v>
       </c>
@@ -5828,7 +5887,7 @@
       <c r="T46" s="5"/>
       <c r="U46" s="8"/>
     </row>
-    <row r="47" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
         <v>246</v>
       </c>
@@ -5884,7 +5943,7 @@
       <c r="T47" s="5"/>
       <c r="U47" s="8"/>
     </row>
-    <row r="48" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
         <v>246</v>
       </c>
@@ -5940,7 +5999,7 @@
       <c r="T48" s="5"/>
       <c r="U48" s="8"/>
     </row>
-    <row r="49" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
         <v>246</v>
       </c>
@@ -5996,7 +6055,7 @@
       <c r="T49" s="5"/>
       <c r="U49" s="8"/>
     </row>
-    <row r="50" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
         <v>395</v>
       </c>
@@ -6049,7 +6108,7 @@
       <c r="T50" s="5"/>
       <c r="U50" s="8"/>
     </row>
-    <row r="51" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
         <v>395</v>
       </c>
@@ -6066,7 +6125,7 @@
         <v>8</v>
       </c>
       <c r="F51" s="5"/>
-      <c r="I51" s="12" t="b">
+      <c r="I51" s="15" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -6094,7 +6153,7 @@
       <c r="T51" s="5"/>
       <c r="U51" s="8"/>
     </row>
-    <row r="52" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
         <v>395</v>
       </c>
@@ -6147,7 +6206,7 @@
       <c r="T52" s="5"/>
       <c r="U52" s="8"/>
     </row>
-    <row r="53" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
         <v>395</v>
       </c>
@@ -6200,7 +6259,7 @@
       <c r="T53" s="5"/>
       <c r="U53" s="8"/>
     </row>
-    <row r="54" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
         <v>420</v>
       </c>
@@ -6250,7 +6309,7 @@
       <c r="T54" s="5"/>
       <c r="U54" s="8"/>
     </row>
-    <row r="55" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
         <v>424</v>
       </c>
@@ -6303,7 +6362,7 @@
       <c r="T55" s="5"/>
       <c r="U55" s="8"/>
     </row>
-    <row r="56" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
         <v>424</v>
       </c>
@@ -6359,7 +6418,7 @@
       <c r="T56" s="5"/>
       <c r="U56" s="8"/>
     </row>
-    <row r="57" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
         <v>424</v>
       </c>
@@ -6412,7 +6471,7 @@
       <c r="T57" s="5"/>
       <c r="U57" s="8"/>
     </row>
-    <row r="58" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
         <v>424</v>
       </c>
@@ -6422,7 +6481,7 @@
       <c r="C58" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="D58" s="11" t="s">
+      <c r="D58" s="14" t="s">
         <v>352</v>
       </c>
       <c r="E58" s="5" t="s">
@@ -6468,7 +6527,7 @@
       <c r="T58" s="5"/>
       <c r="U58" s="8"/>
     </row>
-    <row r="59" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
         <v>424</v>
       </c>
@@ -6524,7 +6583,7 @@
       <c r="T59" s="5"/>
       <c r="U59" s="8"/>
     </row>
-    <row r="60" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
         <v>424</v>
       </c>
@@ -6582,7 +6641,7 @@
       <c r="T60" s="5"/>
       <c r="U60" s="8"/>
     </row>
-    <row r="61" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
         <v>424</v>
       </c>
@@ -6641,7 +6700,7 @@
       <c r="T61" s="5"/>
       <c r="U61" s="8"/>
     </row>
-    <row r="62" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
         <v>424</v>
       </c>
@@ -6750,7 +6809,7 @@
       <c r="T63" s="5"/>
       <c r="U63" s="8"/>
     </row>
-    <row r="64" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
         <v>424</v>
       </c>
@@ -6803,7 +6862,7 @@
       <c r="T64" s="5"/>
       <c r="U64" s="8"/>
     </row>
-    <row r="65" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
         <v>424</v>
       </c>
@@ -6813,7 +6872,7 @@
       <c r="C65" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="D65" s="11" t="s">
+      <c r="D65" s="14" t="s">
         <v>352</v>
       </c>
       <c r="E65" s="5" t="s">
@@ -6864,7 +6923,7 @@
       <c r="T65" s="5"/>
       <c r="U65" s="8"/>
     </row>
-    <row r="66" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
         <v>424</v>
       </c>
@@ -6874,7 +6933,7 @@
       <c r="C66" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="D66" s="11" t="s">
+      <c r="D66" s="14" t="s">
         <v>352</v>
       </c>
       <c r="E66" s="5" t="s">
@@ -6920,7 +6979,7 @@
       <c r="T66" s="5"/>
       <c r="U66" s="8"/>
     </row>
-    <row r="67" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
         <v>424</v>
       </c>
@@ -6979,7 +7038,7 @@
       <c r="T67" s="5"/>
       <c r="U67" s="8"/>
     </row>
-    <row r="68" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
         <v>424</v>
       </c>
@@ -7035,7 +7094,7 @@
       <c r="T68" s="5"/>
       <c r="U68" s="8"/>
     </row>
-    <row r="69" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
         <v>499</v>
       </c>
@@ -7091,7 +7150,7 @@
       <c r="T69" s="5"/>
       <c r="U69" s="8"/>
     </row>
-    <row r="70" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
         <v>510</v>
       </c>
@@ -7149,7 +7208,7 @@
       <c r="T70" s="5"/>
       <c r="U70" s="8"/>
     </row>
-    <row r="71" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
         <v>510</v>
       </c>
@@ -7207,7 +7266,7 @@
       <c r="T71" s="5"/>
       <c r="U71" s="8"/>
     </row>
-    <row r="72" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
         <v>510</v>
       </c>
@@ -7263,7 +7322,7 @@
       <c r="T72" s="5"/>
       <c r="U72" s="8"/>
     </row>
-    <row r="73" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
         <v>510</v>
       </c>
@@ -7324,7 +7383,7 @@
       <c r="T73" s="5"/>
       <c r="U73" s="8"/>
     </row>
-    <row r="74" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
         <v>510</v>
       </c>
@@ -7383,7 +7442,7 @@
       <c r="T74" s="5"/>
       <c r="U74" s="8"/>
     </row>
-    <row r="75" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
         <v>510</v>
       </c>
@@ -7444,7 +7503,7 @@
       <c r="T75" s="5"/>
       <c r="U75" s="8"/>
     </row>
-    <row r="76" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
         <v>510</v>
       </c>
@@ -7502,7 +7561,7 @@
       <c r="T76" s="5"/>
       <c r="U76" s="8"/>
     </row>
-    <row r="77" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
         <v>510</v>
       </c>
@@ -7512,7 +7571,7 @@
       <c r="C77" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D77" s="11" t="s">
+      <c r="D77" s="14" t="s">
         <v>352</v>
       </c>
       <c r="E77" s="5" t="s">
@@ -7560,7 +7619,7 @@
       <c r="T77" s="5"/>
       <c r="U77" s="8"/>
     </row>
-    <row r="78" customFormat="false" ht="44" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
         <v>510</v>
       </c>
@@ -7592,13 +7651,13 @@
       <c r="K78" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="L78" s="13" t="s">
+      <c r="L78" s="16" t="s">
         <v>559</v>
       </c>
       <c r="M78" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="N78" s="13" t="s">
+      <c r="N78" s="16" t="s">
         <v>560</v>
       </c>
       <c r="O78" s="5" t="s">
@@ -7619,7 +7678,7 @@
       <c r="T78" s="5"/>
       <c r="U78" s="8"/>
     </row>
-    <row r="79" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="s">
         <v>510</v>
       </c>
@@ -7678,7 +7737,7 @@
       <c r="T79" s="5"/>
       <c r="U79" s="8"/>
     </row>
-    <row r="80" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="5" t="s">
         <v>510</v>
       </c>
@@ -7737,7 +7796,7 @@
       <c r="T80" s="5"/>
       <c r="U80" s="8"/>
     </row>
-    <row r="81" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="5" t="s">
         <v>510</v>
       </c>
@@ -7796,7 +7855,7 @@
       <c r="T81" s="5"/>
       <c r="U81" s="8"/>
     </row>
-    <row r="82" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="5" t="s">
         <v>581</v>
       </c>
@@ -7851,7 +7910,7 @@
       <c r="T82" s="5"/>
       <c r="U82" s="8"/>
     </row>
-    <row r="83" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="5" t="s">
         <v>591</v>
       </c>
@@ -7904,7 +7963,7 @@
       <c r="T83" s="5"/>
       <c r="U83" s="8"/>
     </row>
-    <row r="84" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="5" t="s">
         <v>591</v>
       </c>
@@ -7960,7 +8019,7 @@
       <c r="T84" s="5"/>
       <c r="U84" s="8"/>
     </row>
-    <row r="85" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="5" t="s">
         <v>581</v>
       </c>
@@ -8019,7 +8078,7 @@
       <c r="T85" s="5"/>
       <c r="U85" s="8"/>
     </row>
-    <row r="86" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="5" t="s">
         <v>581</v>
       </c>
@@ -8078,7 +8137,7 @@
       <c r="T86" s="5"/>
       <c r="U86" s="8"/>
     </row>
-    <row r="87" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="5" t="s">
         <v>581</v>
       </c>
@@ -8134,7 +8193,7 @@
       <c r="T87" s="5"/>
       <c r="U87" s="8"/>
     </row>
-    <row r="88" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="5" t="s">
         <v>581</v>
       </c>
@@ -8190,7 +8249,7 @@
       <c r="T88" s="5"/>
       <c r="U88" s="8"/>
     </row>
-    <row r="89" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="5" t="s">
         <v>499</v>
       </c>
@@ -8243,7 +8302,7 @@
       <c r="T89" s="5"/>
       <c r="U89" s="8"/>
     </row>
-    <row r="90" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="5" t="s">
         <v>499</v>
       </c>
@@ -8296,11 +8355,11 @@
       <c r="T90" s="5"/>
       <c r="U90" s="8"/>
     </row>
-    <row r="91" customFormat="false" ht="44" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="5" t="s">
         <v>499</v>
       </c>
-      <c r="B91" s="14" t="s">
+      <c r="B91" s="17" t="s">
         <v>633</v>
       </c>
       <c r="C91" s="5" t="s">
@@ -8326,7 +8385,7 @@
         <v>108</v>
       </c>
       <c r="L91" s="5"/>
-      <c r="N91" s="13" t="s">
+      <c r="N91" s="16" t="s">
         <v>634</v>
       </c>
       <c r="O91" s="5" t="s">
@@ -8347,7 +8406,7 @@
       <c r="T91" s="5"/>
       <c r="U91" s="8"/>
     </row>
-    <row r="92" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="5" t="s">
         <v>635</v>
       </c>
@@ -8441,7 +8500,7 @@
       <c r="T93" s="5"/>
       <c r="U93" s="8"/>
     </row>
-    <row r="94" customFormat="false" ht="12.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="5" t="s">
         <v>645</v>
       </c>
@@ -8451,7 +8510,7 @@
       <c r="C94" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D94" s="15" t="s">
+      <c r="D94" s="18" t="s">
         <v>646</v>
       </c>
       <c r="E94" s="5" t="s">
@@ -8520,16 +8579,7 @@
       <c r="T95" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:U94">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="line_status"/>
-        <filter val="order_status"/>
-        <filter val="result_status"/>
-        <filter val="status"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A2:U94"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -8546,179 +8596,435 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B86"/>
+  <dimension ref="A1:S86"/>
   <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+    <row r="1" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
         <v>654</v>
       </c>
-      <c r="B1" s="5"/>
-    </row>
-    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="B1" s="0" t="s">
         <v>655</v>
       </c>
-      <c r="B2" s="5"/>
-    </row>
-    <row r="3" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="17" t="s">
+      <c r="C1" s="0" t="s">
         <v>656</v>
       </c>
-      <c r="B3" s="5"/>
-    </row>
-    <row r="4" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
+      <c r="D1" s="0" t="s">
         <v>657</v>
       </c>
-      <c r="B4" s="5"/>
+      <c r="E1" s="0" t="s">
+        <v>658</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>659</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>660</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>661</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>662</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>663</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>664</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>665</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>666</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>667</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>668</v>
+      </c>
+      <c r="P1" s="0" t="s">
+        <v>669</v>
+      </c>
+      <c r="Q1" s="0" t="s">
+        <v>670</v>
+      </c>
+      <c r="R1" s="0" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>672</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>673</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="F2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="H2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="I2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="J2" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="K2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="L2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="M2" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="N2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="O2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="P2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="Q2" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="R2" s="20" t="s">
+        <v>674</v>
+      </c>
+      <c r="S2" s="20" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>676</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>677</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="I3" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="J3" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="L3" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="M3" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="N3" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="O3" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="P3" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="Q3" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="R3" s="20" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>679</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>680</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="H4" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="L4" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="M4" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="N4" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="O4" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="P4" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="Q4" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="R4" s="20" t="s">
+        <v>681</v>
+      </c>
+      <c r="S4" s="20" t="s">
+        <v>682</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
-        <v>658</v>
-      </c>
-      <c r="B5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
-        <v>659</v>
-      </c>
-      <c r="B6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>660</v>
-      </c>
+      <c r="A5" s="0" t="s">
+        <v>683</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>680</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="H5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="K5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="L5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="M5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="N5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="O5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="P5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="Q5" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="R5" s="20" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>685</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>677</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="J6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="K6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="L6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="M6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="N6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="O6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="P6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="Q6" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="R6" s="20" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21"/>
       <c r="B7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>661</v>
-      </c>
+    <row r="8" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21"/>
       <c r="B8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>662</v>
-      </c>
+    <row r="9" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21"/>
       <c r="B9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
-        <v>663</v>
-      </c>
+      <c r="A10" s="21"/>
       <c r="B10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
-        <v>664</v>
-      </c>
+      <c r="A11" s="21"/>
       <c r="B11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
+      <c r="A12" s="21"/>
       <c r="B12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
-        <v>669</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
-        <v>670</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="s">
-        <v>671</v>
-      </c>
+      <c r="A13" s="22"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21"/>
+    </row>
+    <row r="21" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21"/>
+    </row>
+    <row r="22" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21"/>
+    </row>
+    <row r="23" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21"/>
+    </row>
+    <row r="24" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21"/>
+    </row>
+    <row r="25" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21"/>
     </row>
     <row r="26" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="27" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16" t="s">
-        <v>672</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="72.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17" t="s">
-        <v>674</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17" t="s">
-        <v>675</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="100.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17" t="s">
-        <v>676</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17" t="s">
-        <v>677</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="114.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17" t="s">
-        <v>678</v>
-      </c>
+      <c r="A27" s="22"/>
+    </row>
+    <row r="28" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="21"/>
+    </row>
+    <row r="29" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21"/>
+    </row>
+    <row r="30" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21"/>
+    </row>
+    <row r="31" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="21"/>
+    </row>
+    <row r="32" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="21"/>
+    </row>
+    <row r="33" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>